<commit_message>
the two ankle push rods are machined aluminium, not printed
Arm_A and Arm_B - the long bars of the 2-RSU ankle - keep their CAD mass (54.8 / 38.8 g),
get no density override, and stay out of the ratio statistics. The measured file now carries
an `aluminium` list for parts like this, and the sheet shows them grey with ratio 1.0 by
definition, exempt from the PLA-ceiling check.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/aluminium_parts_3dprint_masses.xlsx
+++ b/docs/aluminium_parts_3dprint_masses.xlsx
@@ -79,7 +79,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -111,6 +111,11 @@
         <fgColor rgb="00FFD4A8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9DEE5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -138,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -167,6 +172,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2609,7 +2617,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>E열 기입값은 출력물 사진의 손글씨를 읽어 CAD 부품에 대조한 것 — 초록=확실 · 노랑=보통(A/B 짝 미확정) · 주황=불확실(실물 대조 필요). F열이 46 %를 넘으면 빨강: PLA(1.24)/알루(2.70) 물리 상한 초과 = 오독 또는 오배정.</t>
+          <t>E열 기입값은 출력물 사진의 손글씨를 읽어 CAD 부품에 대조한 것 — 초록=확실 · 노랑=보통(A/B 짝 미확정) · 주황=불확실(실물 대조 필요) · 회색=알루미늄 가공품(CAD 질량 그대로). F열이 46 %를 넘으면 빨강: PLA(1.24)/알루(2.70) 물리 상한 초과 = 오독 또는 오배정.</t>
         </is>
       </c>
     </row>
@@ -3285,12 +3293,18 @@
       <c r="D32" s="8" t="n">
         <v>54.76</v>
       </c>
-      <c r="E32" s="9" t="n"/>
+      <c r="E32" s="14" t="n">
+        <v>54.76</v>
+      </c>
       <c r="F32" s="10">
         <f>IF(E32="","",E32/D32)</f>
         <v/>
       </c>
-      <c r="G32" s="6" t="inlineStr"/>
+      <c r="G32" s="11" t="inlineStr">
+        <is>
+          <t>알루미늄(출력 아님) · AB 푸시로드(긴 바) - 알루미늄 가공품, 출력 아님 (사용자 2026-08-23). CAD 질량 그대로</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="92" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
@@ -3673,12 +3687,18 @@
       <c r="D48" s="8" t="n">
         <v>38.77</v>
       </c>
-      <c r="E48" s="9" t="n"/>
+      <c r="E48" s="14" t="n">
+        <v>38.77</v>
+      </c>
       <c r="F48" s="10">
         <f>IF(E48="","",E48/D48)</f>
         <v/>
       </c>
-      <c r="G48" s="6" t="inlineStr"/>
+      <c r="G48" s="11" t="inlineStr">
+        <is>
+          <t>알루미늄(출력 아님) · AB 푸시로드(긴 바) - 알루미늄 가공품, 출력 아님 (사용자 2026-08-23). CAD 질량 그대로</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="92" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
@@ -4058,7 +4078,7 @@
       <c r="E63" s="13" t="n">
         <v>40.5</v>
       </c>
-      <c r="F63" s="14">
+      <c r="F63" s="15">
         <f>IF(E63="","",E63/D63)</f>
         <v/>
       </c>
@@ -4635,16 +4655,16 @@
       <c r="G86" s="6" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="C87" s="15" t="inlineStr">
+      <c r="C87" s="16" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="D87" s="16">
+      <c r="D87" s="17">
         <f>SUM(D6:D86)</f>
         <v/>
       </c>
-      <c r="E87" s="16">
+      <c r="E87" s="17">
         <f>SUM(E6:E86)</f>
         <v/>
       </c>
@@ -4673,7 +4693,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>링크별 합계 — E열에 측정값을 넣는 대로 자동으로 채워집니다</t>
         </is>
@@ -4716,15 +4736,15 @@
         <f>COUNTIF('알루미늄 부품'!$A$6:$A$86,A4)</f>
         <v/>
       </c>
-      <c r="C4" s="18">
+      <c r="C4" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A4,'알루미늄 부품'!$D$6:$D$86)</f>
         <v/>
       </c>
-      <c r="D4" s="18">
+      <c r="D4" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A4,'알루미늄 부품'!$E$6:$E$86)</f>
         <v/>
       </c>
-      <c r="E4" s="18">
+      <c r="E4" s="19">
         <f>COUNTIFS('알루미늄 부품'!$A$6:$A$86,A4,'알루미늄 부품'!$E$6:$E$86,"&lt;&gt;")</f>
         <v/>
       </c>
@@ -4739,15 +4759,15 @@
         <f>COUNTIF('알루미늄 부품'!$A$6:$A$86,A5)</f>
         <v/>
       </c>
-      <c r="C5" s="18">
+      <c r="C5" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A5,'알루미늄 부품'!$D$6:$D$86)</f>
         <v/>
       </c>
-      <c r="D5" s="18">
+      <c r="D5" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A5,'알루미늄 부품'!$E$6:$E$86)</f>
         <v/>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="19">
         <f>COUNTIFS('알루미늄 부품'!$A$6:$A$86,A5,'알루미늄 부품'!$E$6:$E$86,"&lt;&gt;")</f>
         <v/>
       </c>
@@ -4762,15 +4782,15 @@
         <f>COUNTIF('알루미늄 부품'!$A$6:$A$86,A6)</f>
         <v/>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A6,'알루미늄 부품'!$D$6:$D$86)</f>
         <v/>
       </c>
-      <c r="D6" s="18">
+      <c r="D6" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A6,'알루미늄 부품'!$E$6:$E$86)</f>
         <v/>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="19">
         <f>COUNTIFS('알루미늄 부품'!$A$6:$A$86,A6,'알루미늄 부품'!$E$6:$E$86,"&lt;&gt;")</f>
         <v/>
       </c>
@@ -4785,15 +4805,15 @@
         <f>COUNTIF('알루미늄 부품'!$A$6:$A$86,A7)</f>
         <v/>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A7,'알루미늄 부품'!$D$6:$D$86)</f>
         <v/>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A7,'알루미늄 부품'!$E$6:$E$86)</f>
         <v/>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="19">
         <f>COUNTIFS('알루미늄 부품'!$A$6:$A$86,A7,'알루미늄 부품'!$E$6:$E$86,"&lt;&gt;")</f>
         <v/>
       </c>
@@ -4808,15 +4828,15 @@
         <f>COUNTIF('알루미늄 부품'!$A$6:$A$86,A8)</f>
         <v/>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A8,'알루미늄 부품'!$D$6:$D$86)</f>
         <v/>
       </c>
-      <c r="D8" s="18">
+      <c r="D8" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A8,'알루미늄 부품'!$E$6:$E$86)</f>
         <v/>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="19">
         <f>COUNTIFS('알루미늄 부품'!$A$6:$A$86,A8,'알루미늄 부품'!$E$6:$E$86,"&lt;&gt;")</f>
         <v/>
       </c>
@@ -4831,15 +4851,15 @@
         <f>COUNTIF('알루미늄 부품'!$A$6:$A$86,A9)</f>
         <v/>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A9,'알루미늄 부품'!$D$6:$D$86)</f>
         <v/>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A9,'알루미늄 부품'!$E$6:$E$86)</f>
         <v/>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="19">
         <f>COUNTIFS('알루미늄 부품'!$A$6:$A$86,A9,'알루미늄 부품'!$E$6:$E$86,"&lt;&gt;")</f>
         <v/>
       </c>
@@ -4854,15 +4874,15 @@
         <f>COUNTIF('알루미늄 부품'!$A$6:$A$86,A10)</f>
         <v/>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A10,'알루미늄 부품'!$D$6:$D$86)</f>
         <v/>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A10,'알루미늄 부품'!$E$6:$E$86)</f>
         <v/>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="19">
         <f>COUNTIFS('알루미늄 부품'!$A$6:$A$86,A10,'알루미늄 부품'!$E$6:$E$86,"&lt;&gt;")</f>
         <v/>
       </c>
@@ -4877,15 +4897,15 @@
         <f>COUNTIF('알루미늄 부품'!$A$6:$A$86,A11)</f>
         <v/>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A11,'알루미늄 부품'!$D$6:$D$86)</f>
         <v/>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A11,'알루미늄 부품'!$E$6:$E$86)</f>
         <v/>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="19">
         <f>COUNTIFS('알루미늄 부품'!$A$6:$A$86,A11,'알루미늄 부품'!$E$6:$E$86,"&lt;&gt;")</f>
         <v/>
       </c>
@@ -4900,15 +4920,15 @@
         <f>COUNTIF('알루미늄 부품'!$A$6:$A$86,A12)</f>
         <v/>
       </c>
-      <c r="C12" s="18">
+      <c r="C12" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A12,'알루미늄 부품'!$D$6:$D$86)</f>
         <v/>
       </c>
-      <c r="D12" s="18">
+      <c r="D12" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A12,'알루미늄 부품'!$E$6:$E$86)</f>
         <v/>
       </c>
-      <c r="E12" s="18">
+      <c r="E12" s="19">
         <f>COUNTIFS('알루미늄 부품'!$A$6:$A$86,A12,'알루미늄 부품'!$E$6:$E$86,"&lt;&gt;")</f>
         <v/>
       </c>
@@ -4923,15 +4943,15 @@
         <f>COUNTIF('알루미늄 부품'!$A$6:$A$86,A13)</f>
         <v/>
       </c>
-      <c r="C13" s="18">
+      <c r="C13" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A13,'알루미늄 부품'!$D$6:$D$86)</f>
         <v/>
       </c>
-      <c r="D13" s="18">
+      <c r="D13" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A13,'알루미늄 부품'!$E$6:$E$86)</f>
         <v/>
       </c>
-      <c r="E13" s="18">
+      <c r="E13" s="19">
         <f>COUNTIFS('알루미늄 부품'!$A$6:$A$86,A13,'알루미늄 부품'!$E$6:$E$86,"&lt;&gt;")</f>
         <v/>
       </c>
@@ -4946,15 +4966,15 @@
         <f>COUNTIF('알루미늄 부품'!$A$6:$A$86,A14)</f>
         <v/>
       </c>
-      <c r="C14" s="18">
+      <c r="C14" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A14,'알루미늄 부품'!$D$6:$D$86)</f>
         <v/>
       </c>
-      <c r="D14" s="18">
+      <c r="D14" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A14,'알루미늄 부품'!$E$6:$E$86)</f>
         <v/>
       </c>
-      <c r="E14" s="18">
+      <c r="E14" s="19">
         <f>COUNTIFS('알루미늄 부품'!$A$6:$A$86,A14,'알루미늄 부품'!$E$6:$E$86,"&lt;&gt;")</f>
         <v/>
       </c>
@@ -4969,38 +4989,38 @@
         <f>COUNTIF('알루미늄 부품'!$A$6:$A$86,A15)</f>
         <v/>
       </c>
-      <c r="C15" s="18">
+      <c r="C15" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A15,'알루미늄 부품'!$D$6:$D$86)</f>
         <v/>
       </c>
-      <c r="D15" s="18">
+      <c r="D15" s="19">
         <f>SUMIF('알루미늄 부품'!$A$6:$A$86,A15,'알루미늄 부품'!$E$6:$E$86)</f>
         <v/>
       </c>
-      <c r="E15" s="18">
+      <c r="E15" s="19">
         <f>COUNTIFS('알루미늄 부품'!$A$6:$A$86,A15,'알루미늄 부품'!$E$6:$E$86,"&lt;&gt;")</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="B16" s="19">
+      <c r="B16" s="20">
         <f>SUM(B4:B15)</f>
         <v/>
       </c>
-      <c r="C16" s="20">
+      <c r="C16" s="21">
         <f>SUM(C4:C15)</f>
         <v/>
       </c>
-      <c r="D16" s="20">
+      <c r="D16" s="21">
         <f>SUM(D4:D15)</f>
         <v/>
       </c>
-      <c r="E16" s="20">
+      <c r="E16" s="21">
         <f>SUM(E4:E15)</f>
         <v/>
       </c>

</xml_diff>